<commit_message>
Test hygiene + Data Layer plan (no app code changes)
- Mobile Real Device Test recorded as "Deferred by owner" in reports and Excel
- e2e scripts aligned with the current flow; old-spec expectations reported as
  Obsolete/N/A instead of FAIL (marker selection by point ID, empty-floor note,
  fullscreen v1.7 spec, mobile tap after camera settles, WL-* marker IDs,
  refresh opens building view, lift buttons enabled, "จอดชั้น X", accel window)
- docs/data-layer/DATA-LAYER-PLAN.md: architecture, file list, Fortune migration plan

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LMeWfurV1NvMP1iCPXsbJw
</commit_message>
<xml_diff>
--- a/docs/reports/IoT-Fortune-Performance-GPU.xlsx
+++ b/docs/reports/IoT-Fortune-Performance-GPU.xlsx
@@ -335,7 +335,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="176">
   <si>
     <t xml:space="preserve">สรุปสถานะ Performance — build 194ccdd (feature/adaptive-quality)</t>
   </si>
@@ -400,16 +400,16 @@
     <t xml:space="preserve">Performance</t>
   </si>
   <si>
-    <t xml:space="preserve">Mobile Target</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ยังไม่ได้ตัดสิน</t>
+    <t xml:space="preserve">Mobile Real Device Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deferred by owner</t>
   </si>
   <si>
     <t xml:space="preserve">Mobile ≥ 30 FPS บนมือถือจริง</t>
   </si>
   <si>
-    <t xml:space="preserve">มีเพียง Mobile Viewport Simulation (ไม่ใช่มือถือจริง) — รอวัดบนอุปกรณ์จริง</t>
+    <t xml:space="preserve">Deferred by owner — ยังไม่ได้ทดสอบ ไม่ถือว่าผ่านหรือไม่ผ่าน และต้องทดสอบก่อน Production Release · คู่มือและ Bookmarklet เก็บไว้ที่ docs/reports/MOBILE-REAL-DEVICE-TEST.md และ scripts/perf/ · มีเพียง Mobile Viewport Simulation (ไม่ใช่มือถือจริง)</t>
   </si>
   <si>
     <t xml:space="preserve">Mobile Viewport Simulation</t>
@@ -544,10 +544,20 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">• Mobile Real Device Test: Deferred by owner — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="FreeSans"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">• วัดบนมือถือจริง </t>
+      <t xml:space="preserve">ต้องทดสอบบนมือถือจริง </t>
     </r>
     <r>
       <rPr>
@@ -566,7 +576,7 @@
         <rFont val="FreeSans"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">ก่อนตัดสินเกณฑ์ </t>
+      <t xml:space="preserve">ก่อน </t>
     </r>
     <r>
       <rPr>
@@ -576,10 +586,88 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Mobile</t>
+      <t xml:space="preserve">Production Release</t>
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• เกณฑ์เดินหน้าพัฒนารอบนี้</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ผล </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Desktop GPU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">จริง </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ตัดสินโดยเจ้าของงาน</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Performance บน GPU จริง — build ใหม่ (194ccdd) เทียบ ddc56f0</t>
   </si>
   <si>
@@ -937,7 +1025,10 @@
     <t xml:space="preserve">หลังจบ: ปิดทุก Layer · ทึบ (รอ 30 วิ)</t>
   </si>
   <si>
-    <t xml:space="preserve">• ผลนี้ไม่ใช่ผลมือถือจริง: วัดเพียงผลของจอเล็ก/Layout มือถือบน GPU Desktop — ต้องวัดซ้ำบนมือถือจริง (Android กลาง ๆ และ iPhone) ก่อนตัดสินเกณฑ์ Mobile ≥ 30 FPS</t>
+    <t xml:space="preserve">• ผลนี้ไม่ใช่ผลมือถือจริง: วัดเพียงผลของจอเล็ก/Layout มือถือบน GPU Desktop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Mobile Real Device Test: Deferred by owner — ยังไม่ได้ทดสอบ ไม่ถือว่าผ่านหรือไม่ผ่าน และต้องทดสอบก่อน Production Release</t>
   </si>
   <si>
     <t xml:space="preserve">• Canvas เล็กกว่า Desktop มาก จึงใช้ GPU น้อยกว่า (หนักสุด 10.5 ms เทียบ 16.1 ms บน Desktop)</t>
@@ -1119,7 +1210,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1146,8 +1237,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <fgColor rgb="FFEDEDED"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -1158,14 +1249,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDEDED"/>
-        <bgColor rgb="FFE2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFCE4D6"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFEDEDED"/>
       </patternFill>
     </fill>
   </fills>
@@ -1305,7 +1390,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1317,19 +1402,19 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1374,7 +1459,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF2CC"/>
+      <rgbColor rgb="FFFCE4D6"/>
       <rgbColor rgb="FFDDE7EE"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -1391,7 +1476,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFE2EFDA"/>
-      <rgbColor rgb="FFFCE4D6"/>
+      <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -1597,7 +1682,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -1730,8 +1815,13 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="0" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1770,17 +1860,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>45</v>
@@ -1788,63 +1878,63 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>52.4</v>
@@ -1893,10 +1983,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C7" s="14" t="n">
         <v>51.6</v>
@@ -1945,10 +2035,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>44.9</v>
@@ -1997,10 +2087,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>57</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>56</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>44.8</v>
@@ -2049,10 +2139,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" s="14" t="n">
         <v>34.4</v>
@@ -2103,10 +2193,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C11" s="14" t="n">
         <v>30.8</v>
@@ -2157,24 +2247,24 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2245,37 +2335,37 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -2307,43 +2397,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>3</v>
@@ -2351,10 +2441,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C6" s="16" t="n">
         <v>19</v>
@@ -2370,18 +2460,18 @@
       </c>
       <c r="G6" s="13"/>
       <c r="H6" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C7" s="16" t="n">
         <v>20</v>
@@ -2399,18 +2489,18 @@
         <v>44.8</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>20</v>
@@ -2426,18 +2516,18 @@
       </c>
       <c r="G8" s="13"/>
       <c r="H8" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C9" s="16" t="n">
         <v>20</v>
@@ -2455,15 +2545,15 @@
         <v>46.6</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C11" s="20" t="n">
         <f aca="false">C9-C6</f>
@@ -2484,26 +2574,26 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B15" s="16" t="n">
         <v>1</v>
@@ -2518,7 +2608,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B16" s="16" t="n">
         <v>0</v>
@@ -2533,7 +2623,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B17" s="16" t="n">
         <v>0</v>
@@ -2548,7 +2638,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B18" s="16" t="n">
         <v>1</v>
@@ -2563,7 +2653,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B19" s="16" t="n">
         <v>1</v>
@@ -2578,13 +2668,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D20" s="13" t="str">
         <f aca="false">IF(B20=C20,"ผ่าน","ตรวจต่อ")</f>
@@ -2593,7 +2683,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B21" s="16" t="n">
         <v>0</v>
@@ -2608,7 +2698,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B22" s="16" t="n">
         <v>0</v>
@@ -2623,17 +2713,17 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2675,17 +2765,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B3" s="24" t="n">
         <f aca="false">Performance!B3</f>
@@ -2694,75 +2784,75 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="U5" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
@@ -2797,7 +2887,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C7" s="16" t="n">
         <v>52.7</v>
@@ -2864,7 +2954,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>51.9</v>
@@ -2931,7 +3021,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C9" s="16" t="n">
         <v>53.5</v>
@@ -2998,7 +3088,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C10" s="16" t="n">
         <v>55.8</v>
@@ -3065,7 +3155,7 @@
         <v>5</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C11" s="16" t="n">
         <v>54.6</v>
@@ -3132,7 +3222,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C12" s="16" t="n">
         <v>56.9</v>
@@ -3199,7 +3289,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C13" s="16" t="n">
         <v>55.2</v>
@@ -3266,7 +3356,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>32.7</v>
@@ -3333,7 +3423,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>49.2</v>
@@ -3400,7 +3490,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C16" s="16" t="n">
         <v>56.3</v>
@@ -3464,10 +3554,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
@@ -3499,10 +3589,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>124</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>123</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
@@ -3534,10 +3624,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
@@ -3569,12 +3659,12 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E22" s="30" t="n">
         <f aca="false">AVERAGEIF(T7:T16,"ใช้ได้",C7:C16)</f>
@@ -3583,7 +3673,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E23" s="30" t="n">
         <f aca="false">_xlfn.MINIFS(C7:C16,T7:T16,"ใช้ได้")</f>
@@ -3592,7 +3682,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E24" s="31" t="n">
         <f aca="false">COUNTIF(T7:T16,"&lt;&gt;ใช้ได้")</f>
@@ -3601,7 +3691,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E25" s="30" t="n">
         <f aca="false">MAX(O7:O16)</f>
@@ -3610,7 +3700,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E26" s="30" t="n">
         <f aca="false">AVERAGE(O17:O19)</f>
@@ -3619,7 +3709,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E27" s="20" t="n">
         <f aca="false">E26-O6</f>
@@ -3628,7 +3718,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E28" s="22" t="n">
         <f aca="false">L19-L6</f>
@@ -3637,7 +3727,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E29" s="22" t="n">
         <f aca="false">M19-M6</f>
@@ -3646,7 +3736,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E30" s="22" t="n">
         <f aca="false">N19-N6</f>
@@ -3655,7 +3745,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E31" s="31" t="n">
         <f aca="false">Q19</f>
@@ -3664,12 +3754,12 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
@@ -3677,7 +3767,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>0</v>
@@ -3685,7 +3775,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>0</v>
@@ -3693,7 +3783,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E38" s="32" t="n">
         <v>1</v>
@@ -3701,7 +3791,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E39" s="32" t="n">
         <v>1</v>
@@ -3709,45 +3799,45 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E40" s="32" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="13" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -3766,7 +3856,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -3786,17 +3876,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>30</v>
@@ -3804,66 +3894,66 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B6" s="16" t="n">
         <v>59.3</v>
@@ -3923,7 +4013,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B7" s="16" t="n">
         <v>50.3</v>
@@ -3983,7 +4073,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B8" s="16" t="n">
         <v>48</v>
@@ -4043,7 +4133,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>59.4</v>
@@ -4103,27 +4193,32 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>156</v>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -4152,79 +4247,79 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>